<commit_message>
Populate Modern Times' own Furniture_Rates.xlsx instead of an empty template
Copied Umang's full 39-row rate sheet into Modern Times' own
Furniture_Rates.xlsx (previously just headers) and pointed its config
back at the local file, so it's a real, self-contained, directly-editable
spreadsheet rather than a cross-project reference. Dimensions still read
from Umang's sheet (single source of truth for that data). Verified the
product-card match count is unchanged (29/29) after the switch.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/modern-times/Furniture_Rates.xlsx
+++ b/projects/modern-times/Furniture_Rates.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -463,15 +463,405 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Furniture</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Item Rate</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Barstool 01 B</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Barstool 03</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Barstool 11</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>26000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bed 01 A</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bed 04</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>111000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bed 27 A</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>141000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bed 47</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>98000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Bench 03 A</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bench 14 A</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>47000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bench 20 B</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Centre table 02 A</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Centre Table 13 A</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Centre Table 23</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Chair 06</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Chair 07</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>29000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Chair 12 C</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>26000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Chair 42 A</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>37000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Chair 27 A</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Chair 44 C</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Chair 05</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Chair 09 A</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Dining Table 03</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>72000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Side Table 01</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Side Table 02 A</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Side Table 02 C</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Side Table 08 B</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>31000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Side Table 31 C</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Side Table 42 A</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>28000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Sofa 23</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sofa 28 C</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>106000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Sofa 36 A</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>101000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Storage Unit 16</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>82000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Storage Unit 29 C</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>54000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Storage Unit 34 A</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>82000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Study Table 02 A</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>44000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Study Table 11</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>51000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Swing 04 A</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>77000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TV Unit 09 R2</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TV Unit 29 A R2</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>24000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>